<commit_message>
Put the barley workbook in each section of Describing Data
The chapter had one workbook at the end, after all the statistics had been
taught. Peter's rebuilt Sask_barley_varieties_2025.xlsx has a tab per topic --
Centre, Location, Spread, Histogram -- so each section now embeds it pointing
at its own tab via the ActiveCell parameter.

Removes the trailing "detailed example" section, whose dataset introduction and
stranded box-plot instructions no longer had a place, and drops the two
remaining box-plot references.

The share GUID is a placeholder until the workbook is uploaded.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_conditional.xlsx
+++ b/textbook_examples/mod01_conditional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B8715FB-2E99-954B-814A-3C40060B914A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{0B8715FB-2E99-954B-814A-3C40060B914A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C77AAF20-6382-6C48-9628-02C1E0016A22}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>Conditional functions</t>
   </si>
@@ -107,13 +107,7 @@
     <t>How many yields above 60?</t>
   </si>
   <si>
-    <t>Average wheat yield over 250 ac</t>
-  </si>
-  <si>
-    <t>How many above the average?</t>
-  </si>
-  <si>
-    <t>The last one is the awkward case: the threshold is itself a calculation, so you glue "&gt;" onto it with &amp;.  Quoting the whole thing as "&gt;AVERAGE(...)" would search for that literal text.</t>
+    <t>Average wheat yield in fields over 250 acres</t>
   </si>
 </sst>
 </file>
@@ -220,9 +214,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,15 +525,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="1" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="29.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -755,123 +751,99 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="11"/>
+      <c r="C15" s="7">
         <f>COUNTIF(B5:B12,"Canola")</f>
         <v>3</v>
       </c>
-      <c r="C15" s="12" t="str">
-        <f t="shared" ref="C15:C20" ca="1" si="2">_xlfn.FORMULATEXT(B15)</f>
+      <c r="D15" s="12" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C15)</f>
         <v>=COUNTIF(B5:B12,"Canola")</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="11"/>
+      <c r="C16" s="7">
         <f>SUMIF(B5:B12,"Canola",C5:C12)</f>
         <v>650</v>
       </c>
-      <c r="C16" s="12" t="str">
-        <f t="shared" ca="1" si="2"/>
+      <c r="D16" s="12" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C16)</f>
         <v>=SUMIF(B5:B12,"Canola",C5:C12)</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="11"/>
+      <c r="C17" s="7">
         <f>AVERAGEIF(B5:B12,"Canola",D5:D12)</f>
         <v>41.3</v>
       </c>
-      <c r="C17" s="12" t="str">
-        <f t="shared" ca="1" si="2"/>
+      <c r="D17" s="12" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C17)</f>
         <v>=AVERAGEIF(B5:B12,"Canola",D5:D12)</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="11"/>
+      <c r="C18" s="7">
         <f>COUNTIF(D5:D12,"&gt;60")</f>
         <v>3</v>
       </c>
-      <c r="C18" s="12" t="str">
-        <f t="shared" ca="1" si="2"/>
+      <c r="D18" s="12" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C18)</f>
         <v>=COUNTIF(D5:D12,"&gt;60")</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-    </row>
-    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+    </row>
+    <row r="19" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="13"/>
+      <c r="C19" s="7">
         <f>AVERAGEIFS(D5:D12,B5:B12,"Wheat",C5:C12,"&gt;250")</f>
         <v>58.25</v>
       </c>
-      <c r="C19" s="12" t="str">
-        <f t="shared" ca="1" si="2"/>
+      <c r="D19" s="12" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C19)</f>
         <v>=AVERAGEIFS(D5:D12,B5:B12,"Wheat",C5:C12,"&gt;250")</v>
       </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-    </row>
-    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="7">
-        <f>COUNTIF(D5:D12,"&gt;"&amp;AVERAGE(D5:D12))</f>
-        <v>5</v>
-      </c>
-      <c r="C20" s="12" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v>=COUNTIF(D5:D12,"&gt;"&amp;AVERAGE(D5:D12))</v>
-      </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-    </row>
-    <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-    </row>
-    <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C19:F19"/>
+  <mergeCells count="11">
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D19:F19"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update workbooks edited in Excel
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_conditional.xlsx
+++ b/textbook_examples/mod01_conditional.xlsx
@@ -240,11 +240,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -252,9 +250,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -776,12 +776,12 @@
         <f>COUNTIF(B2:B9,"Canola")</f>
         <v>3</v>
       </c>
-      <c r="D12" s="10" t="str">
+      <c r="D12" s="15" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C12)</f>
         <v>=COUNTIF(B2:B9,"Canola")</v>
       </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
@@ -792,12 +792,12 @@
         <f>SUMIF(B2:B9,"Canola",C2:C9)</f>
         <v>650</v>
       </c>
-      <c r="D13" s="10" t="str">
+      <c r="D13" s="15" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C13)</f>
         <v>=SUMIF(B2:B9,"Canola",C2:C9)</v>
       </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
     </row>
     <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
@@ -808,12 +808,12 @@
         <f>AVERAGEIF(B2:B9,"Canola",D2:D9)</f>
         <v>41.3</v>
       </c>
-      <c r="D14" s="10" t="str">
+      <c r="D14" s="15" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C14)</f>
         <v>=AVERAGEIF(B2:B9,"Canola",D2:D9)</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
@@ -824,12 +824,12 @@
         <f>COUNTIF(D2:D9,"&gt;60")</f>
         <v>3</v>
       </c>
-      <c r="D15" s="10" t="str">
+      <c r="D15" s="15" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C15)</f>
         <v>=COUNTIF(D2:D9,"&gt;60")</v>
       </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
     </row>
     <row r="16" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="s">
@@ -840,26 +840,26 @@
         <f>AVERAGEIFS(D2:D9,B2:B9,"Wheat",C2:C9,"&gt;250")</f>
         <v>58.25</v>
       </c>
-      <c r="D16" s="10" t="str">
+      <c r="D16" s="15" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C16)</f>
         <v>=AVERAGEIFS(D2:D9,B2:B9,"Wheat",C2:C9,"&gt;250")</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
     </row>
     <row r="19" spans="1:6" ht="73" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
@@ -1039,7 +1039,7 @@
         <v>18</v>
       </c>
       <c r="B12" s="12"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
@@ -1048,7 +1048,7 @@
         <v>19</v>
       </c>
       <c r="B13" s="12"/>
-      <c r="C13" s="15"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
@@ -1066,7 +1066,7 @@
         <v>21</v>
       </c>
       <c r="B15" s="12"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="7"/>
-      <c r="D16" s="14"/>
+      <c r="D16" s="10"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1088,13 +1088,13 @@
       <c r="A18" s="1"/>
     </row>
     <row r="19" spans="1:5" ht="73" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>

</xml_diff>